<commit_message>
Daily IST report: add CSV/MD/XLSX
</commit_message>
<xml_diff>
--- a/reports/submissions_daily_matrix.xlsx
+++ b/reports/submissions_daily_matrix.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BP109"/>
+  <dimension ref="A1:BQ109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -496,8 +496,9 @@
     <col width="12" customWidth="1" min="64" max="64"/>
     <col width="12" customWidth="1" min="65" max="65"/>
     <col width="12" customWidth="1" min="66" max="66"/>
-    <col width="13" customWidth="1" min="67" max="67"/>
+    <col width="12" customWidth="1" min="67" max="67"/>
     <col width="13" customWidth="1" min="68" max="68"/>
+    <col width="13" customWidth="1" min="69" max="69"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -831,12 +832,17 @@
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="BO1" s="2" t="inlineStr">
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="BP1" s="2" t="inlineStr">
         <is>
           <t>total_files</t>
         </is>
       </c>
-      <c r="BP1" s="2" t="inlineStr">
+      <c r="BQ1" s="2" t="inlineStr">
         <is>
           <t>unique_days</t>
         </is>
@@ -1048,9 +1054,12 @@
         <v>0</v>
       </c>
       <c r="BO2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP2" t="n">
         <v>12</v>
       </c>
-      <c r="BP2" t="n">
+      <c r="BQ2" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1260,9 +1269,12 @@
         <v>0</v>
       </c>
       <c r="BO3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP3" t="n">
         <v>10</v>
       </c>
-      <c r="BP3" t="n">
+      <c r="BQ3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1472,9 +1484,12 @@
         <v>0</v>
       </c>
       <c r="BO4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP4" t="n">
         <v>40</v>
       </c>
-      <c r="BP4" t="n">
+      <c r="BQ4" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1684,9 +1699,12 @@
         <v>0</v>
       </c>
       <c r="BO5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP5" t="n">
         <v>15</v>
       </c>
-      <c r="BP5" t="n">
+      <c r="BQ5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1896,9 +1914,12 @@
         <v>0</v>
       </c>
       <c r="BO6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP6" t="n">
         <v>19</v>
       </c>
-      <c r="BP6" t="n">
+      <c r="BQ6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2108,9 +2129,12 @@
         <v>0</v>
       </c>
       <c r="BO7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP7" t="n">
         <v>19</v>
       </c>
-      <c r="BP7" t="n">
+      <c r="BQ7" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2320,9 +2344,12 @@
         <v>0</v>
       </c>
       <c r="BO8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP8" t="n">
         <v>32</v>
       </c>
-      <c r="BP8" t="n">
+      <c r="BQ8" t="n">
         <v>32</v>
       </c>
     </row>
@@ -2532,9 +2559,12 @@
         <v>0</v>
       </c>
       <c r="BO9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP9" t="n">
         <v>31</v>
       </c>
-      <c r="BP9" t="n">
+      <c r="BQ9" t="n">
         <v>31</v>
       </c>
     </row>
@@ -2744,9 +2774,12 @@
         <v>0</v>
       </c>
       <c r="BO10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP10" t="n">
         <v>39</v>
       </c>
-      <c r="BP10" t="n">
+      <c r="BQ10" t="n">
         <v>39</v>
       </c>
     </row>
@@ -2956,9 +2989,12 @@
         <v>0</v>
       </c>
       <c r="BO11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP11" t="n">
         <v>29</v>
       </c>
-      <c r="BP11" t="n">
+      <c r="BQ11" t="n">
         <v>29</v>
       </c>
     </row>
@@ -3168,9 +3204,12 @@
         <v>0</v>
       </c>
       <c r="BO12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP12" t="n">
         <v>37</v>
       </c>
-      <c r="BP12" t="n">
+      <c r="BQ12" t="n">
         <v>37</v>
       </c>
     </row>
@@ -3380,9 +3419,12 @@
         <v>0</v>
       </c>
       <c r="BO13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP13" t="n">
         <v>14</v>
       </c>
-      <c r="BP13" t="n">
+      <c r="BQ13" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3592,9 +3634,12 @@
         <v>0</v>
       </c>
       <c r="BO14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP14" t="n">
         <v>26</v>
       </c>
-      <c r="BP14" t="n">
+      <c r="BQ14" t="n">
         <v>26</v>
       </c>
     </row>
@@ -3804,9 +3849,12 @@
         <v>0</v>
       </c>
       <c r="BO15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP15" t="n">
         <v>9</v>
       </c>
-      <c r="BP15" t="n">
+      <c r="BQ15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4016,9 +4064,12 @@
         <v>0</v>
       </c>
       <c r="BO16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP16" t="n">
         <v>20</v>
       </c>
-      <c r="BP16" t="n">
+      <c r="BQ16" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4228,9 +4279,12 @@
         <v>0</v>
       </c>
       <c r="BO17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP17" t="n">
         <v>17</v>
       </c>
-      <c r="BP17" t="n">
+      <c r="BQ17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4440,9 +4494,12 @@
         <v>0</v>
       </c>
       <c r="BO18" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP18" t="n">
         <v>33</v>
       </c>
-      <c r="BP18" t="n">
+      <c r="BQ18" t="n">
         <v>33</v>
       </c>
     </row>
@@ -4657,6 +4714,9 @@
       <c r="BP19" t="n">
         <v>0</v>
       </c>
+      <c r="BQ19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4864,9 +4924,12 @@
         <v>0</v>
       </c>
       <c r="BO20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP20" t="n">
         <v>20</v>
       </c>
-      <c r="BP20" t="n">
+      <c r="BQ20" t="n">
         <v>20</v>
       </c>
     </row>
@@ -5076,9 +5139,12 @@
         <v>0</v>
       </c>
       <c r="BO21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP21" t="n">
         <v>27</v>
       </c>
-      <c r="BP21" t="n">
+      <c r="BQ21" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5293,6 +5359,9 @@
       <c r="BP22" t="n">
         <v>0</v>
       </c>
+      <c r="BQ22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5500,9 +5569,12 @@
         <v>0</v>
       </c>
       <c r="BO23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP23" t="n">
         <v>22</v>
       </c>
-      <c r="BP23" t="n">
+      <c r="BQ23" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5712,9 +5784,12 @@
         <v>0</v>
       </c>
       <c r="BO24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP24" t="n">
         <v>27</v>
       </c>
-      <c r="BP24" t="n">
+      <c r="BQ24" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5924,9 +5999,12 @@
         <v>0</v>
       </c>
       <c r="BO25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP25" t="n">
         <v>11</v>
       </c>
-      <c r="BP25" t="n">
+      <c r="BQ25" t="n">
         <v>11</v>
       </c>
     </row>
@@ -6136,9 +6214,12 @@
         <v>0</v>
       </c>
       <c r="BO26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP26" t="n">
         <v>35</v>
       </c>
-      <c r="BP26" t="n">
+      <c r="BQ26" t="n">
         <v>35</v>
       </c>
     </row>
@@ -6348,9 +6429,12 @@
         <v>0</v>
       </c>
       <c r="BO27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP27" t="n">
         <v>25</v>
       </c>
-      <c r="BP27" t="n">
+      <c r="BQ27" t="n">
         <v>23</v>
       </c>
     </row>
@@ -6560,9 +6644,12 @@
         <v>0</v>
       </c>
       <c r="BO28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP28" t="n">
         <v>19</v>
       </c>
-      <c r="BP28" t="n">
+      <c r="BQ28" t="n">
         <v>19</v>
       </c>
     </row>
@@ -6772,9 +6859,12 @@
         <v>0</v>
       </c>
       <c r="BO29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP29" t="n">
         <v>11</v>
       </c>
-      <c r="BP29" t="n">
+      <c r="BQ29" t="n">
         <v>11</v>
       </c>
     </row>
@@ -6984,9 +7074,12 @@
         <v>0</v>
       </c>
       <c r="BO30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP30" t="n">
         <v>25</v>
       </c>
-      <c r="BP30" t="n">
+      <c r="BQ30" t="n">
         <v>25</v>
       </c>
     </row>
@@ -7196,9 +7289,12 @@
         <v>0</v>
       </c>
       <c r="BO31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP31" t="n">
         <v>20</v>
       </c>
-      <c r="BP31" t="n">
+      <c r="BQ31" t="n">
         <v>20</v>
       </c>
     </row>
@@ -7408,9 +7504,12 @@
         <v>0</v>
       </c>
       <c r="BO32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP32" t="n">
         <v>23</v>
       </c>
-      <c r="BP32" t="n">
+      <c r="BQ32" t="n">
         <v>23</v>
       </c>
     </row>
@@ -7620,9 +7719,12 @@
         <v>0</v>
       </c>
       <c r="BO33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP33" t="n">
         <v>21</v>
       </c>
-      <c r="BP33" t="n">
+      <c r="BQ33" t="n">
         <v>21</v>
       </c>
     </row>
@@ -7832,9 +7934,12 @@
         <v>0</v>
       </c>
       <c r="BO34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP34" t="n">
         <v>9</v>
       </c>
-      <c r="BP34" t="n">
+      <c r="BQ34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -8044,9 +8149,12 @@
         <v>0</v>
       </c>
       <c r="BO35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP35" t="n">
         <v>25</v>
       </c>
-      <c r="BP35" t="n">
+      <c r="BQ35" t="n">
         <v>25</v>
       </c>
     </row>
@@ -8256,9 +8364,12 @@
         <v>0</v>
       </c>
       <c r="BO36" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP36" t="n">
         <v>16</v>
       </c>
-      <c r="BP36" t="n">
+      <c r="BQ36" t="n">
         <v>16</v>
       </c>
     </row>
@@ -8473,6 +8584,9 @@
       <c r="BP37" t="n">
         <v>0</v>
       </c>
+      <c r="BQ37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8680,9 +8794,12 @@
         <v>0</v>
       </c>
       <c r="BO38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP38" t="n">
         <v>2</v>
       </c>
-      <c r="BP38" t="n">
+      <c r="BQ38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8892,9 +9009,12 @@
         <v>0</v>
       </c>
       <c r="BO39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP39" t="n">
         <v>37</v>
       </c>
-      <c r="BP39" t="n">
+      <c r="BQ39" t="n">
         <v>37</v>
       </c>
     </row>
@@ -9104,9 +9224,12 @@
         <v>0</v>
       </c>
       <c r="BO40" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP40" t="n">
         <v>28</v>
       </c>
-      <c r="BP40" t="n">
+      <c r="BQ40" t="n">
         <v>28</v>
       </c>
     </row>
@@ -9316,9 +9439,12 @@
         <v>0</v>
       </c>
       <c r="BO41" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP41" t="n">
         <v>39</v>
       </c>
-      <c r="BP41" t="n">
+      <c r="BQ41" t="n">
         <v>39</v>
       </c>
     </row>
@@ -9528,9 +9654,12 @@
         <v>0</v>
       </c>
       <c r="BO42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP42" t="n">
         <v>21</v>
       </c>
-      <c r="BP42" t="n">
+      <c r="BQ42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9740,9 +9869,12 @@
         <v>0</v>
       </c>
       <c r="BO43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP43" t="n">
         <v>60</v>
       </c>
-      <c r="BP43" t="n">
+      <c r="BQ43" t="n">
         <v>19</v>
       </c>
     </row>
@@ -9952,9 +10084,12 @@
         <v>0</v>
       </c>
       <c r="BO44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP44" t="n">
         <v>25</v>
       </c>
-      <c r="BP44" t="n">
+      <c r="BQ44" t="n">
         <v>25</v>
       </c>
     </row>
@@ -10164,9 +10299,12 @@
         <v>0</v>
       </c>
       <c r="BO45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP45" t="n">
         <v>26</v>
       </c>
-      <c r="BP45" t="n">
+      <c r="BQ45" t="n">
         <v>26</v>
       </c>
     </row>
@@ -10376,9 +10514,12 @@
         <v>0</v>
       </c>
       <c r="BO46" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP46" t="n">
         <v>30</v>
       </c>
-      <c r="BP46" t="n">
+      <c r="BQ46" t="n">
         <v>30</v>
       </c>
     </row>
@@ -10593,6 +10734,9 @@
       <c r="BP47" t="n">
         <v>0</v>
       </c>
+      <c r="BQ47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -10800,9 +10944,12 @@
         <v>0</v>
       </c>
       <c r="BO48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP48" t="n">
         <v>27</v>
       </c>
-      <c r="BP48" t="n">
+      <c r="BQ48" t="n">
         <v>27</v>
       </c>
     </row>
@@ -11012,9 +11159,12 @@
         <v>0</v>
       </c>
       <c r="BO49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP49" t="n">
         <v>19</v>
       </c>
-      <c r="BP49" t="n">
+      <c r="BQ49" t="n">
         <v>19</v>
       </c>
     </row>
@@ -11224,9 +11374,12 @@
         <v>0</v>
       </c>
       <c r="BO50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP50" t="n">
         <v>7</v>
       </c>
-      <c r="BP50" t="n">
+      <c r="BQ50" t="n">
         <v>7</v>
       </c>
     </row>
@@ -11436,9 +11589,12 @@
         <v>0</v>
       </c>
       <c r="BO51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP51" t="n">
         <v>32</v>
       </c>
-      <c r="BP51" t="n">
+      <c r="BQ51" t="n">
         <v>32</v>
       </c>
     </row>
@@ -11653,6 +11809,9 @@
       <c r="BP52" t="n">
         <v>0</v>
       </c>
+      <c r="BQ52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -11860,9 +12019,12 @@
         <v>0</v>
       </c>
       <c r="BO53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP53" t="n">
         <v>13</v>
       </c>
-      <c r="BP53" t="n">
+      <c r="BQ53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -12077,6 +12239,9 @@
       <c r="BP54" t="n">
         <v>0</v>
       </c>
+      <c r="BQ54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -12284,9 +12449,12 @@
         <v>0</v>
       </c>
       <c r="BO55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP55" t="n">
         <v>36</v>
       </c>
-      <c r="BP55" t="n">
+      <c r="BQ55" t="n">
         <v>36</v>
       </c>
     </row>
@@ -12496,9 +12664,12 @@
         <v>0</v>
       </c>
       <c r="BO56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP56" t="n">
         <v>31</v>
       </c>
-      <c r="BP56" t="n">
+      <c r="BQ56" t="n">
         <v>31</v>
       </c>
     </row>
@@ -12708,9 +12879,12 @@
         <v>0</v>
       </c>
       <c r="BO57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP57" t="n">
         <v>10</v>
       </c>
-      <c r="BP57" t="n">
+      <c r="BQ57" t="n">
         <v>10</v>
       </c>
     </row>
@@ -12920,9 +13094,12 @@
         <v>0</v>
       </c>
       <c r="BO58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP58" t="n">
         <v>13</v>
       </c>
-      <c r="BP58" t="n">
+      <c r="BQ58" t="n">
         <v>13</v>
       </c>
     </row>
@@ -13132,9 +13309,12 @@
         <v>0</v>
       </c>
       <c r="BO59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP59" t="n">
         <v>6</v>
       </c>
-      <c r="BP59" t="n">
+      <c r="BQ59" t="n">
         <v>6</v>
       </c>
     </row>
@@ -13349,6 +13529,9 @@
       <c r="BP60" t="n">
         <v>0</v>
       </c>
+      <c r="BQ60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -13556,9 +13739,12 @@
         <v>0</v>
       </c>
       <c r="BO61" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP61" t="n">
         <v>29</v>
       </c>
-      <c r="BP61" t="n">
+      <c r="BQ61" t="n">
         <v>29</v>
       </c>
     </row>
@@ -13768,9 +13954,12 @@
         <v>0</v>
       </c>
       <c r="BO62" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP62" t="n">
         <v>29</v>
       </c>
-      <c r="BP62" t="n">
+      <c r="BQ62" t="n">
         <v>29</v>
       </c>
     </row>
@@ -13980,9 +14169,12 @@
         <v>0</v>
       </c>
       <c r="BO63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP63" t="n">
         <v>12</v>
       </c>
-      <c r="BP63" t="n">
+      <c r="BQ63" t="n">
         <v>12</v>
       </c>
     </row>
@@ -14197,6 +14389,9 @@
       <c r="BP64" t="n">
         <v>0</v>
       </c>
+      <c r="BQ64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -14404,9 +14599,12 @@
         <v>0</v>
       </c>
       <c r="BO65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP65" t="n">
         <v>17</v>
       </c>
-      <c r="BP65" t="n">
+      <c r="BQ65" t="n">
         <v>17</v>
       </c>
     </row>
@@ -14616,9 +14814,12 @@
         <v>0</v>
       </c>
       <c r="BO66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP66" t="n">
         <v>8</v>
       </c>
-      <c r="BP66" t="n">
+      <c r="BQ66" t="n">
         <v>8</v>
       </c>
     </row>
@@ -14828,9 +15029,12 @@
         <v>0</v>
       </c>
       <c r="BO67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP67" t="n">
         <v>40</v>
       </c>
-      <c r="BP67" t="n">
+      <c r="BQ67" t="n">
         <v>40</v>
       </c>
     </row>
@@ -15040,9 +15244,12 @@
         <v>0</v>
       </c>
       <c r="BO68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP68" t="n">
         <v>23</v>
       </c>
-      <c r="BP68" t="n">
+      <c r="BQ68" t="n">
         <v>22</v>
       </c>
     </row>
@@ -15252,9 +15459,12 @@
         <v>0</v>
       </c>
       <c r="BO69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP69" t="n">
         <v>7</v>
       </c>
-      <c r="BP69" t="n">
+      <c r="BQ69" t="n">
         <v>7</v>
       </c>
     </row>
@@ -15464,9 +15674,12 @@
         <v>0</v>
       </c>
       <c r="BO70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP70" t="n">
         <v>23</v>
       </c>
-      <c r="BP70" t="n">
+      <c r="BQ70" t="n">
         <v>11</v>
       </c>
     </row>
@@ -15676,9 +15889,12 @@
         <v>0</v>
       </c>
       <c r="BO71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP71" t="n">
         <v>24</v>
       </c>
-      <c r="BP71" t="n">
+      <c r="BQ71" t="n">
         <v>24</v>
       </c>
     </row>
@@ -15888,9 +16104,12 @@
         <v>0</v>
       </c>
       <c r="BO72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP72" t="n">
         <v>24</v>
       </c>
-      <c r="BP72" t="n">
+      <c r="BQ72" t="n">
         <v>24</v>
       </c>
     </row>
@@ -16105,6 +16324,9 @@
       <c r="BP73" t="n">
         <v>0</v>
       </c>
+      <c r="BQ73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -16317,6 +16539,9 @@
       <c r="BP74" t="n">
         <v>0</v>
       </c>
+      <c r="BQ74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -16524,9 +16749,12 @@
         <v>0</v>
       </c>
       <c r="BO75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP75" t="n">
         <v>25</v>
       </c>
-      <c r="BP75" t="n">
+      <c r="BQ75" t="n">
         <v>25</v>
       </c>
     </row>
@@ -16736,9 +16964,12 @@
         <v>0</v>
       </c>
       <c r="BO76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP76" t="n">
         <v>21</v>
       </c>
-      <c r="BP76" t="n">
+      <c r="BQ76" t="n">
         <v>21</v>
       </c>
     </row>
@@ -16948,9 +17179,12 @@
         <v>0</v>
       </c>
       <c r="BO77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP77" t="n">
         <v>15</v>
       </c>
-      <c r="BP77" t="n">
+      <c r="BQ77" t="n">
         <v>15</v>
       </c>
     </row>
@@ -17160,9 +17394,12 @@
         <v>0</v>
       </c>
       <c r="BO78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP78" t="n">
         <v>36</v>
       </c>
-      <c r="BP78" t="n">
+      <c r="BQ78" t="n">
         <v>35</v>
       </c>
     </row>
@@ -17372,9 +17609,12 @@
         <v>0</v>
       </c>
       <c r="BO79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP79" t="n">
         <v>22</v>
       </c>
-      <c r="BP79" t="n">
+      <c r="BQ79" t="n">
         <v>22</v>
       </c>
     </row>
@@ -17584,9 +17824,12 @@
         <v>0</v>
       </c>
       <c r="BO80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP80" t="n">
         <v>12</v>
       </c>
-      <c r="BP80" t="n">
+      <c r="BQ80" t="n">
         <v>12</v>
       </c>
     </row>
@@ -17796,9 +18039,12 @@
         <v>0</v>
       </c>
       <c r="BO81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP81" t="n">
         <v>4</v>
       </c>
-      <c r="BP81" t="n">
+      <c r="BQ81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -18008,9 +18254,12 @@
         <v>0</v>
       </c>
       <c r="BO82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP82" t="n">
         <v>18</v>
       </c>
-      <c r="BP82" t="n">
+      <c r="BQ82" t="n">
         <v>18</v>
       </c>
     </row>
@@ -18220,9 +18469,12 @@
         <v>0</v>
       </c>
       <c r="BO83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP83" t="n">
         <v>17</v>
       </c>
-      <c r="BP83" t="n">
+      <c r="BQ83" t="n">
         <v>17</v>
       </c>
     </row>
@@ -18432,9 +18684,12 @@
         <v>0</v>
       </c>
       <c r="BO84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP84" t="n">
         <v>13</v>
       </c>
-      <c r="BP84" t="n">
+      <c r="BQ84" t="n">
         <v>13</v>
       </c>
     </row>
@@ -18644,9 +18899,12 @@
         <v>0</v>
       </c>
       <c r="BO85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP85" t="n">
         <v>7</v>
       </c>
-      <c r="BP85" t="n">
+      <c r="BQ85" t="n">
         <v>7</v>
       </c>
     </row>
@@ -18861,6 +19119,9 @@
       <c r="BP86" t="n">
         <v>0</v>
       </c>
+      <c r="BQ86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -19068,9 +19329,12 @@
         <v>0</v>
       </c>
       <c r="BO87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP87" t="n">
         <v>19</v>
       </c>
-      <c r="BP87" t="n">
+      <c r="BQ87" t="n">
         <v>19</v>
       </c>
     </row>
@@ -19285,6 +19549,9 @@
       <c r="BP88" t="n">
         <v>0</v>
       </c>
+      <c r="BQ88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -19492,9 +19759,12 @@
         <v>0</v>
       </c>
       <c r="BO89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP89" t="n">
         <v>18</v>
       </c>
-      <c r="BP89" t="n">
+      <c r="BQ89" t="n">
         <v>18</v>
       </c>
     </row>
@@ -19704,9 +19974,12 @@
         <v>0</v>
       </c>
       <c r="BO90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP90" t="n">
         <v>17</v>
       </c>
-      <c r="BP90" t="n">
+      <c r="BQ90" t="n">
         <v>17</v>
       </c>
     </row>
@@ -19916,9 +20189,12 @@
         <v>0</v>
       </c>
       <c r="BO91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP91" t="n">
         <v>42</v>
       </c>
-      <c r="BP91" t="n">
+      <c r="BQ91" t="n">
         <v>13</v>
       </c>
     </row>
@@ -20128,9 +20404,12 @@
         <v>0</v>
       </c>
       <c r="BO92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP92" t="n">
         <v>7</v>
       </c>
-      <c r="BP92" t="n">
+      <c r="BQ92" t="n">
         <v>7</v>
       </c>
     </row>
@@ -20345,6 +20624,9 @@
       <c r="BP93" t="n">
         <v>0</v>
       </c>
+      <c r="BQ93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -20552,9 +20834,12 @@
         <v>0</v>
       </c>
       <c r="BO94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP94" t="n">
         <v>16</v>
       </c>
-      <c r="BP94" t="n">
+      <c r="BQ94" t="n">
         <v>16</v>
       </c>
     </row>
@@ -20764,9 +21049,12 @@
         <v>0</v>
       </c>
       <c r="BO95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP95" t="n">
         <v>7</v>
       </c>
-      <c r="BP95" t="n">
+      <c r="BQ95" t="n">
         <v>7</v>
       </c>
     </row>
@@ -20976,9 +21264,12 @@
         <v>0</v>
       </c>
       <c r="BO96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP96" t="n">
         <v>24</v>
       </c>
-      <c r="BP96" t="n">
+      <c r="BQ96" t="n">
         <v>24</v>
       </c>
     </row>
@@ -21193,6 +21484,9 @@
       <c r="BP97" t="n">
         <v>0</v>
       </c>
+      <c r="BQ97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -21400,9 +21694,12 @@
         <v>0</v>
       </c>
       <c r="BO98" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP98" t="n">
         <v>35</v>
       </c>
-      <c r="BP98" t="n">
+      <c r="BQ98" t="n">
         <v>35</v>
       </c>
     </row>
@@ -21612,9 +21909,12 @@
         <v>0</v>
       </c>
       <c r="BO99" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP99" t="n">
         <v>14</v>
       </c>
-      <c r="BP99" t="n">
+      <c r="BQ99" t="n">
         <v>14</v>
       </c>
     </row>
@@ -21829,6 +22129,9 @@
       <c r="BP100" t="n">
         <v>0</v>
       </c>
+      <c r="BQ100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -22036,9 +22339,12 @@
         <v>1</v>
       </c>
       <c r="BO101" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP101" t="n">
         <v>32</v>
       </c>
-      <c r="BP101" t="n">
+      <c r="BQ101" t="n">
         <v>32</v>
       </c>
     </row>
@@ -22248,9 +22554,12 @@
         <v>0</v>
       </c>
       <c r="BO102" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP102" t="n">
         <v>31</v>
       </c>
-      <c r="BP102" t="n">
+      <c r="BQ102" t="n">
         <v>31</v>
       </c>
     </row>
@@ -22460,9 +22769,12 @@
         <v>0</v>
       </c>
       <c r="BO103" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP103" t="n">
         <v>34</v>
       </c>
-      <c r="BP103" t="n">
+      <c r="BQ103" t="n">
         <v>34</v>
       </c>
     </row>
@@ -22672,9 +22984,12 @@
         <v>0</v>
       </c>
       <c r="BO104" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP104" t="n">
         <v>12</v>
       </c>
-      <c r="BP104" t="n">
+      <c r="BQ104" t="n">
         <v>12</v>
       </c>
     </row>
@@ -22884,9 +23199,12 @@
         <v>0</v>
       </c>
       <c r="BO105" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP105" t="n">
         <v>28</v>
       </c>
-      <c r="BP105" t="n">
+      <c r="BQ105" t="n">
         <v>28</v>
       </c>
     </row>
@@ -23096,9 +23414,12 @@
         <v>0</v>
       </c>
       <c r="BO106" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP106" t="n">
         <v>7</v>
       </c>
-      <c r="BP106" t="n">
+      <c r="BQ106" t="n">
         <v>7</v>
       </c>
     </row>
@@ -23308,9 +23629,12 @@
         <v>0</v>
       </c>
       <c r="BO107" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP107" t="n">
         <v>13</v>
       </c>
-      <c r="BP107" t="n">
+      <c r="BQ107" t="n">
         <v>13</v>
       </c>
     </row>
@@ -23520,9 +23844,12 @@
         <v>0</v>
       </c>
       <c r="BO108" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP108" t="n">
         <v>2</v>
       </c>
-      <c r="BP108" t="n">
+      <c r="BQ108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -23732,9 +24059,12 @@
         <v>0</v>
       </c>
       <c r="BO109" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP109" t="n">
         <v>4</v>
       </c>
-      <c r="BP109" t="n">
+      <c r="BQ109" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>